<commit_message>
Update eclat_habitos_compra notebook to reset execution counts to null and modify dataset path for improved data handling. Replace df_procesado.xlsx with an updated version.
</commit_message>
<xml_diff>
--- a/df_procesado.xlsx
+++ b/df_procesado.xlsx
@@ -3477,11 +3477,7 @@
           <t>Supermercado  (Exito, Jumbo, Etc)</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>1200k</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -5399,11 +5395,7 @@
           <t>Tienda de Barrio</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>700k</t>
-        </is>
-      </c>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -6121,11 +6113,7 @@
           <t>Hard Discount  (D1, ARA, etc )</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>1500k</t>
-        </is>
-      </c>
+      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -15003,11 +14991,7 @@
           <t>Tienda de Barrio</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>1700k</t>
-        </is>
-      </c>
+      <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -18605,11 +18589,7 @@
           <t>Hard Discount  (D1, ARA, etc )</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>500k</t>
-        </is>
-      </c>
+      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -21487,11 +21467,7 @@
           <t xml:space="preserve">Plaza de mercado </t>
         </is>
       </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>1.000.000</t>
-        </is>
-      </c>
+      <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -21729,11 +21705,7 @@
           <t>Hard Discount  (D1, ARA, etc )</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>1000k</t>
-        </is>
-      </c>
+      <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -22211,11 +22183,7 @@
           <t>Hard Discount  (D1, ARA, etc )</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>700k</t>
-        </is>
-      </c>
+      <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -23173,11 +23141,7 @@
           <t>Supermercado  (Exito, Jumbo, Etc)</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>1200k</t>
-        </is>
-      </c>
+      <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -23655,11 +23619,7 @@
           <t>Hard Discount  (D1, ARA, etc )</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>1000k</t>
-        </is>
-      </c>
+      <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -24377,11 +24337,7 @@
           <t>Hard Discount  (D1, ARA, etc )</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>600k</t>
-        </is>
-      </c>
+      <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
           <t>Adulto joven</t>
@@ -35179,11 +35135,7 @@
           <t>Supermercado  (Exito, Jumbo, Etc)</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>2000k</t>
-        </is>
-      </c>
+      <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -36381,11 +36333,7 @@
           <t>Supermercado  (Exito, Jumbo, Etc)</t>
         </is>
       </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>1000k</t>
-        </is>
-      </c>
+      <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -37583,11 +37531,7 @@
           <t>Supermercado  (Exito, Jumbo, Etc)</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>1800k</t>
-        </is>
-      </c>
+      <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
           <t>Joven</t>
@@ -39745,11 +39689,7 @@
           <t>Hard Discount  (D1, ARA, etc )</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr">
-        <is>
-          <t>1500k</t>
-        </is>
-      </c>
+      <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr">
         <is>
           <t>Joven</t>

</xml_diff>

<commit_message>
Update eclat_habitos_compra notebook with revised age bins and labels for demographic analysis. Enhanced Markdown documentation to provide detailed descriptions of dataset variables. Replace df_procesado.xlsx with an updated version for improved data handling.
</commit_message>
<xml_diff>
--- a/df_procesado.xlsx
+++ b/df_procesado.xlsx
@@ -837,7 +837,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -3442,7 +3442,7 @@
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M14" t="n">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -4390,7 +4390,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Adulto</t>
+          <t>31-60</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -5336,7 +5336,7 @@
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -5573,7 +5573,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -5810,7 +5810,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -6045,7 +6045,7 @@
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M26" t="n">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M27" t="n">
@@ -6993,7 +6993,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M28" t="n">
@@ -7230,7 +7230,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M29" t="n">
@@ -7467,7 +7467,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M30" t="n">
@@ -7704,7 +7704,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M31" t="n">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M33" t="n">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M34" t="n">
@@ -8652,7 +8652,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M35" t="n">
@@ -8889,7 +8889,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M36" t="n">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M37" t="n">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Adulto joven</t>
+          <t>26-30</t>
         </is>
       </c>
       <c r="M38" t="n">
@@ -9600,7 +9600,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M39" t="n">
@@ -9837,7 +9837,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M40" t="n">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M41" t="n">
@@ -10311,7 +10311,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M42" t="n">
@@ -10548,7 +10548,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M43" t="n">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M44" t="n">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -11259,7 +11259,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M46" t="n">
@@ -11496,7 +11496,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -11733,7 +11733,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M48" t="n">
@@ -11970,7 +11970,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M49" t="n">
@@ -12207,7 +12207,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M50" t="n">
@@ -12444,7 +12444,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M51" t="n">
@@ -12681,7 +12681,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M52" t="n">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M53" t="n">
@@ -13155,7 +13155,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M54" t="n">
@@ -13392,7 +13392,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M55" t="n">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M56" t="n">
@@ -13866,7 +13866,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M57" t="n">
@@ -14103,7 +14103,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M58" t="n">
@@ -14340,7 +14340,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M59" t="n">
@@ -14577,7 +14577,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M60" t="n">
@@ -14812,7 +14812,7 @@
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M61" t="n">
@@ -15049,7 +15049,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Adulto joven</t>
+          <t>26-30</t>
         </is>
       </c>
       <c r="M62" t="n">
@@ -15286,7 +15286,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M63" t="n">
@@ -15523,7 +15523,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M64" t="n">
@@ -15760,7 +15760,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M65" t="n">
@@ -15997,7 +15997,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M66" t="n">
@@ -16234,7 +16234,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M67" t="n">
@@ -16471,7 +16471,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M68" t="n">
@@ -16708,7 +16708,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M69" t="n">
@@ -16945,7 +16945,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M70" t="n">
@@ -17182,7 +17182,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M71" t="n">
@@ -17419,7 +17419,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M72" t="n">
@@ -17656,7 +17656,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M73" t="n">
@@ -17893,7 +17893,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M74" t="n">
@@ -18130,7 +18130,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M75" t="n">
@@ -18365,7 +18365,7 @@
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M76" t="n">
@@ -18602,7 +18602,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M77" t="n">
@@ -18839,7 +18839,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M78" t="n">
@@ -19076,7 +19076,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M79" t="n">
@@ -19313,7 +19313,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M80" t="n">
@@ -19550,7 +19550,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M81" t="n">
@@ -19787,7 +19787,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M82" t="n">
@@ -20024,7 +20024,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M83" t="n">
@@ -20261,7 +20261,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M84" t="n">
@@ -20498,7 +20498,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M85" t="n">
@@ -20735,7 +20735,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M86" t="n">
@@ -20972,7 +20972,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M87" t="n">
@@ -21207,7 +21207,7 @@
       <c r="K88" t="inlineStr"/>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M88" t="n">
@@ -21442,7 +21442,7 @@
       <c r="K89" t="inlineStr"/>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M89" t="n">
@@ -21679,7 +21679,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M90" t="n">
@@ -21914,7 +21914,7 @@
       <c r="K91" t="inlineStr"/>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M91" t="n">
@@ -22151,7 +22151,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M92" t="n">
@@ -22388,7 +22388,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M93" t="n">
@@ -22625,7 +22625,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M94" t="n">
@@ -22860,7 +22860,7 @@
       <c r="K95" t="inlineStr"/>
       <c r="L95" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M95" t="n">
@@ -23097,7 +23097,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M96" t="n">
@@ -23332,7 +23332,7 @@
       <c r="K97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M97" t="n">
@@ -23569,7 +23569,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M98" t="n">
@@ -23806,7 +23806,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M99" t="n">
@@ -24041,7 +24041,7 @@
       <c r="K100" t="inlineStr"/>
       <c r="L100" t="inlineStr">
         <is>
-          <t>Adulto joven</t>
+          <t>26-30</t>
         </is>
       </c>
       <c r="M100" t="n">
@@ -24278,7 +24278,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M101" t="n">
@@ -24515,7 +24515,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M102" t="n">
@@ -24752,7 +24752,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M103" t="n">
@@ -24989,7 +24989,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M104" t="n">
@@ -25226,7 +25226,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M105" t="n">
@@ -25463,7 +25463,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M106" t="n">
@@ -25700,7 +25700,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M107" t="n">
@@ -25937,7 +25937,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M108" t="n">
@@ -26174,7 +26174,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M109" t="n">
@@ -26411,7 +26411,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M110" t="n">
@@ -26648,7 +26648,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M111" t="n">
@@ -26885,7 +26885,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M112" t="n">
@@ -27122,7 +27122,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M113" t="n">
@@ -27359,7 +27359,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M114" t="n">
@@ -27596,7 +27596,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M115" t="n">
@@ -27833,7 +27833,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M116" t="n">
@@ -28070,7 +28070,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M117" t="n">
@@ -28307,7 +28307,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M118" t="n">
@@ -28544,7 +28544,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M119" t="n">
@@ -28781,7 +28781,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M120" t="n">
@@ -29018,7 +29018,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M121" t="n">
@@ -29255,7 +29255,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M122" t="n">
@@ -29492,7 +29492,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M123" t="n">
@@ -29729,7 +29729,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M124" t="n">
@@ -29966,7 +29966,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M125" t="n">
@@ -30203,7 +30203,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M126" t="n">
@@ -30440,7 +30440,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M127" t="n">
@@ -30677,7 +30677,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M128" t="n">
@@ -30914,7 +30914,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M129" t="n">
@@ -31151,7 +31151,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M130" t="n">
@@ -31388,7 +31388,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M131" t="n">
@@ -31625,7 +31625,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M132" t="n">
@@ -31862,7 +31862,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M133" t="n">
@@ -32099,7 +32099,7 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M134" t="n">
@@ -32336,7 +32336,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M135" t="n">
@@ -32573,7 +32573,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M136" t="n">
@@ -32810,7 +32810,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M137" t="n">
@@ -33047,7 +33047,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M138" t="n">
@@ -33284,7 +33284,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M139" t="n">
@@ -33521,7 +33521,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M140" t="n">
@@ -33758,7 +33758,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M141" t="n">
@@ -33995,7 +33995,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M142" t="n">
@@ -34232,7 +34232,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M143" t="n">
@@ -34469,7 +34469,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M144" t="n">
@@ -34704,7 +34704,7 @@
       <c r="K145" t="inlineStr"/>
       <c r="L145" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M145" t="n">
@@ -34941,7 +34941,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M146" t="n">
@@ -35178,7 +35178,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M147" t="n">
@@ -35415,7 +35415,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M148" t="n">
@@ -35652,7 +35652,7 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M149" t="n">
@@ -35887,7 +35887,7 @@
       <c r="K150" t="inlineStr"/>
       <c r="L150" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M150" t="n">
@@ -36124,7 +36124,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M151" t="n">
@@ -36361,7 +36361,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M152" t="n">
@@ -36598,7 +36598,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M153" t="n">
@@ -36835,7 +36835,7 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M154" t="n">
@@ -37070,7 +37070,7 @@
       <c r="K155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M155" t="n">
@@ -37307,7 +37307,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M156" t="n">
@@ -37544,7 +37544,7 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M157" t="n">
@@ -37781,7 +37781,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M158" t="n">
@@ -38018,7 +38018,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M159" t="n">
@@ -38255,7 +38255,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M160" t="n">
@@ -38492,7 +38492,7 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M161" t="n">
@@ -38729,7 +38729,7 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M162" t="n">
@@ -38966,7 +38966,7 @@
       </c>
       <c r="L163" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M163" t="n">
@@ -39201,7 +39201,7 @@
       <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M164" t="n">
@@ -39438,7 +39438,7 @@
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M165" t="n">
@@ -39675,7 +39675,7 @@
       </c>
       <c r="L166" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M166" t="n">
@@ -39912,7 +39912,7 @@
       </c>
       <c r="L167" t="inlineStr">
         <is>
-          <t>Adulto joven</t>
+          <t>26-30</t>
         </is>
       </c>
       <c r="M167" t="n">
@@ -40149,7 +40149,7 @@
       </c>
       <c r="L168" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M168" t="n">
@@ -40386,7 +40386,7 @@
       </c>
       <c r="L169" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M169" t="n">
@@ -40623,7 +40623,7 @@
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>Menor de 18</t>
         </is>
       </c>
       <c r="M170" t="n">
@@ -40860,7 +40860,7 @@
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M171" t="n">
@@ -41097,7 +41097,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M172" t="n">
@@ -41334,7 +41334,7 @@
       </c>
       <c r="L173" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M173" t="n">
@@ -41571,7 +41571,7 @@
       </c>
       <c r="L174" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M174" t="n">
@@ -41808,7 +41808,7 @@
       </c>
       <c r="L175" t="inlineStr">
         <is>
-          <t>Adulto joven</t>
+          <t>26-30</t>
         </is>
       </c>
       <c r="M175" t="n">
@@ -42045,7 +42045,7 @@
       </c>
       <c r="L176" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M176" t="n">
@@ -42282,7 +42282,7 @@
       </c>
       <c r="L177" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M177" t="n">
@@ -42519,7 +42519,7 @@
       </c>
       <c r="L178" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M178" t="n">
@@ -42756,7 +42756,7 @@
       </c>
       <c r="L179" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M179" t="n">
@@ -42993,7 +42993,7 @@
       </c>
       <c r="L180" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M180" t="n">
@@ -43230,7 +43230,7 @@
       </c>
       <c r="L181" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M181" t="n">
@@ -43467,7 +43467,7 @@
       </c>
       <c r="L182" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M182" t="n">
@@ -43704,7 +43704,7 @@
       </c>
       <c r="L183" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M183" t="n">
@@ -43941,7 +43941,7 @@
       </c>
       <c r="L184" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M184" t="n">
@@ -44178,7 +44178,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M185" t="n">
@@ -44415,7 +44415,7 @@
       </c>
       <c r="L186" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M186" t="n">
@@ -44652,7 +44652,7 @@
       </c>
       <c r="L187" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M187" t="n">
@@ -44889,7 +44889,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M188" t="n">
@@ -45126,7 +45126,7 @@
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M189" t="n">
@@ -45363,7 +45363,7 @@
       </c>
       <c r="L190" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M190" t="n">
@@ -45600,7 +45600,7 @@
       </c>
       <c r="L191" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M191" t="n">
@@ -45837,7 +45837,7 @@
       </c>
       <c r="L192" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M192" t="n">
@@ -46074,7 +46074,7 @@
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M193" t="n">
@@ -46311,7 +46311,7 @@
       </c>
       <c r="L194" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M194" t="n">
@@ -46548,7 +46548,7 @@
       </c>
       <c r="L195" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M195" t="n">
@@ -46785,7 +46785,7 @@
       </c>
       <c r="L196" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M196" t="n">
@@ -47022,7 +47022,7 @@
       </c>
       <c r="L197" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M197" t="n">
@@ -47259,7 +47259,7 @@
       </c>
       <c r="L198" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M198" t="n">
@@ -47496,7 +47496,7 @@
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M199" t="n">
@@ -47733,7 +47733,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M200" t="n">
@@ -47970,7 +47970,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>Joven</t>
+          <t>18-25</t>
         </is>
       </c>
       <c r="M201" t="n">

</xml_diff>